<commit_message>
Backup QR Scanner data - 2026-03-09T08:50:44.278Z - Cache Bust: 1773046244278
</commit_message>
<xml_diff>
--- a/log_history/Y1_B2526_Pharmacology_scanner1773040350333_4791e799a156631a1e6528d73ff0b32fbeeb62851b63d680bacede618e9287f5.xlsx
+++ b/log_history/Y1_B2526_Pharmacology_scanner1773040350333_4791e799a156631a1e6528d73ff0b32fbeeb62851b63d680bacede618e9287f5.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Session" sheetId="1" r:id="rId1"/>
+    <sheet name="Pharmacology" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F58"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1079,9 +1079,489 @@
         <v>marian.samir@med.asu.edu.eg</v>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>254443</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C35" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="D35" t="str">
+        <v>10:12:10</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F35" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>254437</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C36" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="D36" t="str">
+        <v>10:12:10</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F36" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>254417</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C37" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="D37" t="str">
+        <v>10:13:32</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Manual</v>
+      </c>
+      <c r="F37" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>254379</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C38" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="D38" t="str">
+        <v>10:13:37</v>
+      </c>
+      <c r="E38" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F38" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>244495</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C39" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="D39" t="str">
+        <v>10:14:06</v>
+      </c>
+      <c r="E39" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F39" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>254425</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C40" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="D40" t="str">
+        <v>10:14:22</v>
+      </c>
+      <c r="E40" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F40" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>254384</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C41" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="D41" t="str">
+        <v>10:14:28</v>
+      </c>
+      <c r="E41" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F41" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>254369</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C42" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="D42" t="str">
+        <v>10:14:38</v>
+      </c>
+      <c r="E42" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F42" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>254370</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C43" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="D43" t="str">
+        <v>10:14:45</v>
+      </c>
+      <c r="E43" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F43" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>254368</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C44" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="D44" t="str">
+        <v>10:14:50</v>
+      </c>
+      <c r="E44" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F44" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>254358</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C45" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="D45" t="str">
+        <v>10:14:53</v>
+      </c>
+      <c r="E45" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F45" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>254413</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C46" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="D46" t="str">
+        <v>10:15:22</v>
+      </c>
+      <c r="E46" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F46" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>254507</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C47" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="D47" t="str">
+        <v>10:15:35</v>
+      </c>
+      <c r="E47" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F47" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>254390</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C48" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="D48" t="str">
+        <v>10:15:50</v>
+      </c>
+      <c r="E48" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F48" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>254445</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C49" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="D49" t="str">
+        <v>10:15:56</v>
+      </c>
+      <c r="E49" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F49" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>254380</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C50" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="D50" t="str">
+        <v>10:16:05</v>
+      </c>
+      <c r="E50" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F50" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>254441</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C51" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="D51" t="str">
+        <v>10:16:11</v>
+      </c>
+      <c r="E51" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F51" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>254421</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C52" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="D52" t="str">
+        <v>10:16:16</v>
+      </c>
+      <c r="E52" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F52" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>254486</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C53" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="D53" t="str">
+        <v>10:16:23</v>
+      </c>
+      <c r="E53" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F53" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>254364</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C54" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="D54" t="str">
+        <v>10:16:28</v>
+      </c>
+      <c r="E54" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F54" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>254449</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C55" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="D55" t="str">
+        <v>10:16:32</v>
+      </c>
+      <c r="E55" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F55" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>254363</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C56" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="D56" t="str">
+        <v>10:16:46</v>
+      </c>
+      <c r="E56" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F56" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>254389</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C57" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="D57" t="str">
+        <v>10:16:51</v>
+      </c>
+      <c r="E57" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F57" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>254356</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C58" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="D58" t="str">
+        <v>10:18:06</v>
+      </c>
+      <c r="E58" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F58" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F34"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F58"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>